<commit_message>
update list observation code 1a2121ab223f1699eff04c9c89f66868f284db16
</commit_message>
<xml_diff>
--- a/ig/nr-add-nos-generate-profil-table/observations-summary.xlsx
+++ b/ig/nr-add-nos-generate-profil-table/observations-summary.xlsx
@@ -182,7 +182,7 @@
     <t>Nombre de pas par jour</t>
   </si>
   <si>
-    <t>null#41950-7</t>
+    <t>LOINC#41950-7</t>
   </si>
   <si>
     <t>mesures-observation-waist-circumference</t>
@@ -835,7 +835,7 @@
         <v>56</v>
       </c>
       <c r="F15" t="s" s="2">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G15" t="s" s="2">
         <v>17</v>

</xml_diff>

<commit_message>
add FR Profile (#89) 8cd28d7b3e43b67079d83619775a15371f9aa029
</commit_message>
<xml_diff>
--- a/ig/nr-add-nos-generate-profil-table/observations-summary.xlsx
+++ b/ig/nr-add-nos-generate-profil-table/observations-summary.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="63">
   <si>
     <t>Profile</t>
   </si>
@@ -144,6 +144,15 @@
   </si>
   <si>
     <t>null#2708-6</t>
+  </si>
+  <si>
+    <t>mesures-fr-observation-resp-rate</t>
+  </si>
+  <si>
+    <t>Fréquence respiratoire</t>
+  </si>
+  <si>
+    <t>null#9279-1</t>
   </si>
   <si>
     <t>mesures-observation-glucose</t>
@@ -325,7 +334,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -727,16 +736,16 @@
         <v>14</v>
       </c>
       <c r="E12" t="s" s="2">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="F12" t="s" s="2">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="G12" t="s" s="2">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="H12" t="s" s="2">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="I12" t="s" s="2">
         <v>19</v>
@@ -750,25 +759,25 @@
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
+        <v>47</v>
+      </c>
+      <c r="B13" t="s" s="2">
         <v>48</v>
       </c>
-      <c r="B13" t="s" s="2">
+      <c r="C13" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="D13" t="s" s="2">
+        <v>14</v>
+      </c>
+      <c r="E13" t="s" s="2">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s" s="2">
         <v>49</v>
       </c>
-      <c r="C13" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="D13" t="s" s="2">
-        <v>14</v>
-      </c>
-      <c r="E13" t="s" s="2">
+      <c r="G13" t="s" s="2">
         <v>50</v>
-      </c>
-      <c r="F13" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="G13" t="s" s="2">
-        <v>17</v>
       </c>
       <c r="H13" t="s" s="2">
         <v>23</v>
@@ -803,7 +812,7 @@
         <v>16</v>
       </c>
       <c r="G14" t="s" s="2">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="H14" t="s" s="2">
         <v>23</v>
@@ -838,7 +847,7 @@
         <v>16</v>
       </c>
       <c r="G15" t="s" s="2">
-        <v>17</v>
+        <v>50</v>
       </c>
       <c r="H15" t="s" s="2">
         <v>23</v>
@@ -885,6 +894,41 @@
         <v>14</v>
       </c>
       <c r="K16" t="s" s="2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="2">
+        <v>60</v>
+      </c>
+      <c r="B17" t="s" s="2">
+        <v>61</v>
+      </c>
+      <c r="C17" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="D17" t="s" s="2">
+        <v>14</v>
+      </c>
+      <c r="E17" t="s" s="2">
+        <v>62</v>
+      </c>
+      <c r="F17" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="G17" t="s" s="2">
+        <v>17</v>
+      </c>
+      <c r="H17" t="s" s="2">
+        <v>23</v>
+      </c>
+      <c r="I17" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="J17" t="s" s="2">
+        <v>14</v>
+      </c>
+      <c r="K17" t="s" s="2">
         <v>14</v>
       </c>
     </row>

</xml_diff>